<commit_message>
debut de logique backend en cours..
</commit_message>
<xml_diff>
--- a/public/apprenants-model.xlsx
+++ b/public/apprenants-model.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Nom</t>
   </si>
@@ -32,40 +32,31 @@
     <t>Prénom</t>
   </si>
   <si>
-    <t>Apprenant 1</t>
-  </si>
-  <si>
-    <t>Classe</t>
-  </si>
-  <si>
-    <t>Terminale</t>
-  </si>
-  <si>
-    <t>Serie</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Sexe</t>
   </si>
   <si>
     <t>Masculin</t>
   </si>
   <si>
-    <t>Apprenant 2</t>
-  </si>
-  <si>
     <t>Féminin</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>MAMRE</t>
-  </si>
-  <si>
     <t>Parent(phone)</t>
+  </si>
+  <si>
+    <t>ZINSSOU</t>
+  </si>
+  <si>
+    <t>Aime</t>
+  </si>
+  <si>
+    <t>KOCOU</t>
+  </si>
+  <si>
+    <t>Viviane</t>
+  </si>
+  <si>
+    <t>ID Classe</t>
   </si>
 </sst>
 </file>
@@ -122,12 +113,9 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="7">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -161,15 +149,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:F2" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="A1:F2"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Nom" dataDxfId="5"/>
-    <tableColumn id="2" name="Prénom" dataDxfId="4"/>
-    <tableColumn id="5" name="Parent(phone)" dataDxfId="3"/>
-    <tableColumn id="6" name="Serie" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:E2" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E2"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Nom" dataDxfId="4"/>
+    <tableColumn id="2" name="Prénom" dataDxfId="3"/>
+    <tableColumn id="5" name="Parent(phone)" dataDxfId="2"/>
     <tableColumn id="3" name="Sexe" dataDxfId="1"/>
-    <tableColumn id="4" name="Classe" dataDxfId="0"/>
+    <tableColumn id="4" name="ID Classe" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -438,18 +425,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="1"/>
     <col min="2" max="2" width="16.6328125" style="1" customWidth="1"/>
     <col min="3" max="3" width="25.54296875" style="1" customWidth="1"/>
-    <col min="4" max="5" width="21.90625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="33.36328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="22.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.90625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.36328125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,56 +444,47 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="C2" s="3">
+        <v>22956854390</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="E2" s="4">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3">
-        <v>2233</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="3" t="s">
+    <row r="3" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="3">
-        <v>2295681</v>
+        <v>22956854391</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="4" t="s">
         <v>4</v>
+      </c>
+      <c r="E3" s="4">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>